<commit_message>
3.0.17 implement objectClassDeclare. if true, class keyword is replaced with object.
</commit_message>
<xml_diff>
--- a/meta/program/BlancoCgClassValueObject.xlsx
+++ b/meta/program/BlancoCgClassValueObject.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tueda/data/webstorm/blanco/blancoCg/meta/program/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDC4211A-55E2-1349-A6DD-F7961CFFF18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAC559FA-B78E-A14B-87BD-C1CF26CEE8B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21140" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="91">
   <si>
     <t>バリューオブジェクト定義書</t>
   </si>
@@ -458,6 +458,23 @@
     <t>primary constructor に JsonCreator アノテーションを付与します。</t>
     <rPh sb="42" eb="44">
       <t xml:space="preserve">フヨシマス。 </t>
+    </rPh>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>objectClassDeclare</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>trueの場合、class に代えて object でクラス宣言を行います。</t>
+    <rPh sb="5" eb="7">
+      <t xml:space="preserve">バアイ </t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t xml:space="preserve">カワッテ </t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t xml:space="preserve">オコナイマス </t>
     </rPh>
     <phoneticPr fontId="4"/>
   </si>
@@ -953,44 +970,44 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1010,9 +1027,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 テーマ">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1050,7 +1067,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1156,7 +1173,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1298,7 +1315,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1309,7 +1326,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -1374,12 +1391,12 @@
         <v>12</v>
       </c>
       <c r="B8" s="6"/>
-      <c r="C8" s="48" t="s">
+      <c r="C8" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="49"/>
-      <c r="E8" s="49"/>
-      <c r="F8" s="50"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="48"/>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="16" t="s">
@@ -1480,23 +1497,23 @@
       <c r="F18"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="42" t="s">
+      <c r="A19" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="43" t="s">
+      <c r="B19" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="51"/>
+      <c r="C19" s="45"/>
+      <c r="D19" s="45"/>
+      <c r="E19" s="49"/>
       <c r="F19"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="42"/>
-      <c r="B20" s="43"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="51"/>
+      <c r="A20" s="53"/>
+      <c r="B20" s="54"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="49"/>
       <c r="F20"/>
     </row>
     <row r="21" spans="1:6">
@@ -1533,29 +1550,29 @@
       <c r="F24" s="6"/>
     </row>
     <row r="25" spans="1:6" ht="13.5" customHeight="1">
-      <c r="A25" s="42" t="s">
+      <c r="A25" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="42" t="s">
+      <c r="B25" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="45" t="s">
+      <c r="C25" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="D25" s="45" t="s">
+      <c r="D25" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="E25" s="45" t="s">
+      <c r="E25" s="44" t="s">
         <v>6</v>
       </c>
       <c r="F25" s="28"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="42"/>
-      <c r="B26" s="42"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
+      <c r="A26" s="53"/>
+      <c r="B26" s="53"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="44"/>
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:6" ht="33.75" customHeight="1">
@@ -1569,10 +1586,10 @@
         <v>46</v>
       </c>
       <c r="D27" s="19"/>
-      <c r="E27" s="52" t="s">
+      <c r="E27" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="F27" s="53"/>
+      <c r="F27" s="51"/>
     </row>
     <row r="28" spans="1:6" ht="29.25" customHeight="1">
       <c r="A28" s="20">
@@ -1586,14 +1603,14 @@
         <v>46</v>
       </c>
       <c r="D28" s="22"/>
-      <c r="E28" s="54" t="s">
+      <c r="E28" s="52" t="s">
         <v>50</v>
       </c>
-      <c r="F28" s="47"/>
+      <c r="F28" s="43"/>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="20">
-        <f t="shared" ref="A29:A44" si="0">A28+1</f>
+        <f t="shared" ref="A29:A45" si="0">A28+1</f>
         <v>3</v>
       </c>
       <c r="B29" s="21" t="s">
@@ -1622,10 +1639,10 @@
       <c r="D30" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="46" t="s">
+      <c r="E30" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="F30" s="47"/>
+      <c r="F30" s="43"/>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="20">
@@ -1660,10 +1677,10 @@
       <c r="D32" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="E32" s="46" t="s">
+      <c r="E32" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="F32" s="47"/>
+      <c r="F32" s="43"/>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="20">
@@ -1705,6 +1722,7 @@
     </row>
     <row r="35" spans="1:6" ht="42" customHeight="1">
       <c r="A35" s="20">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B35" s="21" t="s">
@@ -1716,13 +1734,14 @@
       <c r="D35" s="41" t="s">
         <v>79</v>
       </c>
-      <c r="E35" s="46" t="s">
+      <c r="E35" s="42" t="s">
         <v>81</v>
       </c>
-      <c r="F35" s="47"/>
+      <c r="F35" s="43"/>
     </row>
     <row r="36" spans="1:6" ht="29.25" customHeight="1">
       <c r="A36" s="20">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B36" s="21" t="s">
@@ -1734,13 +1753,14 @@
       <c r="D36" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="E36" s="46" t="s">
+      <c r="E36" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="F36" s="47"/>
+      <c r="F36" s="43"/>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="20">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B37" s="21" t="s">
@@ -1759,6 +1779,7 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="20">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B38" s="21" t="s">
@@ -1777,6 +1798,7 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="20">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B39" s="21" t="s">
@@ -1812,41 +1834,41 @@
       </c>
       <c r="F40" s="23"/>
     </row>
-    <row r="41" spans="1:6" ht="44.25" customHeight="1">
+    <row r="41" spans="1:6">
       <c r="A41" s="20">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="D41" s="22"/>
-      <c r="E41" s="46" t="s">
-        <v>59</v>
-      </c>
-      <c r="F41" s="47"/>
-    </row>
-    <row r="42" spans="1:6" ht="35" customHeight="1">
+        <v>85</v>
+      </c>
+      <c r="D41" s="22" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F41" s="23"/>
+    </row>
+    <row r="42" spans="1:6" ht="44.25" customHeight="1">
       <c r="A42" s="20">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>77</v>
+        <v>45</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="D42" s="22" t="s">
-        <v>70</v>
-      </c>
-      <c r="E42" s="46" t="s">
-        <v>76</v>
-      </c>
-      <c r="F42" s="47"/>
+        <v>48</v>
+      </c>
+      <c r="D42" s="22"/>
+      <c r="E42" s="42" t="s">
+        <v>59</v>
+      </c>
+      <c r="F42" s="43"/>
     </row>
     <row r="43" spans="1:6" ht="35" customHeight="1">
       <c r="A43" s="20">
@@ -1854,18 +1876,18 @@
         <v>17</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D43" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="E43" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="F43" s="47"/>
+        <v>70</v>
+      </c>
+      <c r="E43" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="F43" s="43"/>
     </row>
     <row r="44" spans="1:6" ht="35" customHeight="1">
       <c r="A44" s="20">
@@ -1873,31 +1895,56 @@
         <v>18</v>
       </c>
       <c r="B44" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="C44" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D44" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="E44" s="42" t="s">
+        <v>83</v>
+      </c>
+      <c r="F44" s="43"/>
+    </row>
+    <row r="45" spans="1:6" ht="35" customHeight="1">
+      <c r="A45" s="20">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="B45" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C44" s="22" t="s">
+      <c r="C45" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D44" s="22" t="b">
+      <c r="D45" s="22" t="b">
         <v>0</v>
       </c>
-      <c r="E44" s="46" t="s">
+      <c r="E45" s="42" t="s">
         <v>88</v>
       </c>
-      <c r="F44" s="47"/>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45" s="24"/>
-      <c r="B45" s="25"/>
-      <c r="C45" s="26"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="27"/>
+      <c r="F45" s="43"/>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="24"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="E45:F45"/>
     <mergeCell ref="E44:F44"/>
-    <mergeCell ref="E43:F43"/>
     <mergeCell ref="D25:D26"/>
     <mergeCell ref="D19:D20"/>
     <mergeCell ref="C8:F8"/>
@@ -1905,22 +1952,16 @@
     <mergeCell ref="E25:E26"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E43:F43"/>
     <mergeCell ref="E42:F42"/>
-    <mergeCell ref="E41:F41"/>
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="E36:F36"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
   </mergeCells>
   <phoneticPr fontId="4"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D61" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D62" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>型</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>